<commit_message>
Sort dataset deterministically so CV folds do not depend on workbook row order
</commit_message>
<xml_diff>
--- a/stacked_model/results/ablation/ablation_summary.xlsx
+++ b/stacked_model/results/ablation/ablation_summary.xlsx
@@ -462,13 +462,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>90.33897607891215</v>
+        <v>90.26621989035854</v>
       </c>
       <c r="C2" t="n">
-        <v>6.359699350431534</v>
+        <v>6.339640638339641</v>
       </c>
       <c r="D2" t="n">
-        <v>5.045117675946887</v>
+        <v>5.134302522274557</v>
       </c>
       <c r="E2" t="n">
         <v>10</v>
@@ -481,16 +481,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>89.88189545145596</v>
+        <v>89.88189012993664</v>
       </c>
       <c r="C3" t="n">
-        <v>7.196125543096576</v>
+        <v>7.053171890746228</v>
       </c>
       <c r="D3" t="n">
-        <v>5.609290932497315</v>
+        <v>5.60929093249731</v>
       </c>
       <c r="E3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -500,13 +500,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>90.26622160524404</v>
+        <v>90.14480748109477</v>
       </c>
       <c r="C4" t="n">
-        <v>6.500918123022267</v>
+        <v>6.576584393800755</v>
       </c>
       <c r="D4" t="n">
-        <v>5.13430252227456</v>
+        <v>5.291435146034402</v>
       </c>
       <c r="E4" t="n">
         <v>9</v>
@@ -519,13 +519,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>91.16121756469221</v>
+        <v>91.16123663287607</v>
       </c>
       <c r="C5" t="n">
-        <v>3.838739020630698</v>
+        <v>3.566841645327663</v>
       </c>
       <c r="D5" t="n">
-        <v>3.281514021417501</v>
+        <v>3.281514021417506</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -538,10 +538,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>90.85719869579637</v>
+        <v>90.85719869579707</v>
       </c>
       <c r="C6" t="n">
-        <v>8.372071372961212</v>
+        <v>8.372071372960381</v>
       </c>
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">

</xml_diff>